<commit_message>
Apply suggestion from @sga-esante 7840d421009df23787706201369875b3d6d84ecc
</commit_message>
<xml_diff>
--- a/sg-rorquestionnaire/ig/StructureDefinition-ror-launchcontext.xlsx
+++ b/sg-rorquestionnaire/ig/StructureDefinition-ror-launchcontext.xlsx
@@ -42,7 +42,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>Profil de LaunchContextExtension créée dans le cadre du ROR afin d'ajouter le name 'structure' acceptant les ressources FHIR 'Organization', 'HealthcareService' et 'Location'</t>
+    <t>Profil de LaunchContextExtension créée dans le cadre du ROR afin d'ajouter le name 'ror-structure' acceptant les ressources FHIR 'Organization', 'HealthcareService' et 'Location'</t>
   </si>
   <si>
     <t>Status</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-13T15:04:48+00:00</t>
+    <t>2026-02-13T15:15:54+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>